<commit_message>
Taller 1 administrativo al viernes 23 de octubre, 8:00, en paralelo con el comercial
Cronograma, sesiones y citaciones con la fecha nueva; vista por semanas
corregida para los talleres 1 y el T2 comercial; brief de José, ajustes y
propuesta con las fechas del 19 de octubre.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ja1vbRoiAwxTq3mLFGrVau
</commit_message>
<xml_diff>
--- a/docentes/administrativo/Sesiones de Teams · perfil administrativo.xlsx
+++ b/docentes/administrativo/Sesiones de Teams · perfil administrativo.xlsx
@@ -477,7 +477,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>18 reuniones · encuentros miércoles de 8:00 a 9:30 a.m. · consultorio de 4:00 a 5:00 p.m. · cronograma ajustado del 15 de octubre de 2026</t>
+          <t>18 reuniones · encuentros miércoles de 8:00 a 9:30 a.m. (Taller 1: viernes 23 de octubre a la misma hora) · consultorio de 4:00 a 5:00 p.m. · cronograma ajustado del 19 de octubre de 2026</t>
         </is>
       </c>
     </row>
@@ -549,12 +549,12 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>21/10/2026</t>
+          <t>23/10/2026</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>miércoles 21 de octubre</t>
+          <t>viernes 23 de octubre</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
@@ -600,12 +600,12 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>23/10/2026</t>
+          <t>27/10/2026</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>viernes 23 de octubre</t>
+          <t>martes 27 de octubre</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">

</xml_diff>